<commit_message>
Se agrega modificacion de features en base a lineas con combinaciones de datos desde datadriven
</commit_message>
<xml_diff>
--- a/tests/automatizacion api/serenity rest/src/test/resources/datadriven/datadriven.xlsx
+++ b/tests/automatizacion api/serenity rest/src/test/resources/datadriven/datadriven.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jherrodr\Downloads\EverestAutomatizacion\demo-servicios-axet-plugin\tests\automatizacion api\serenity rest\src\test\resources\datadriven\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C099BAF-A054-4B41-83C1-B7A9E9C15A07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBA3B66E-31A8-4185-AEE9-B1AB98FA9915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C8F6870A-3E76-401C-B9AA-EF83B2FD7DC2}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{C8F6870A-3E76-401C-B9AA-EF83B2FD7DC2}"/>
   </bookViews>
   <sheets>
     <sheet name="retiro" sheetId="4" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="111">
   <si>
     <t>banco</t>
   </si>
@@ -299,9 +299,6 @@
     <t>pago_factura.operacionobj.AcctBal[1].CurAmt.CurCode</t>
   </si>
   <si>
-    <t>consulta_factura</t>
-  </si>
-  <si>
     <t>bbogota</t>
   </si>
   <si>
@@ -323,9 +320,6 @@
     <t>KR 11 # 71 -73</t>
   </si>
   <si>
-    <t>pago_factura</t>
-  </si>
-  <si>
     <t>PAGO_FACTURA</t>
   </si>
   <si>
@@ -369,6 +363,18 @@
   </si>
   <si>
     <t>PAGO_OBLIGACIONES</t>
+  </si>
+  <si>
+    <t>tipo_request_detalle</t>
+  </si>
+  <si>
+    <t>consulta</t>
+  </si>
+  <si>
+    <t>recaudo</t>
+  </si>
+  <si>
+    <t>1,00028E+13</t>
   </si>
 </sst>
 </file>
@@ -412,9 +418,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -749,7 +756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E55F708-9DF7-49A1-960F-B30120907588}">
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
@@ -919,6 +926,148 @@
         <v>1245</v>
       </c>
     </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3">
+        <v>7946</v>
+      </c>
+      <c r="G3">
+        <v>6032</v>
+      </c>
+      <c r="H3">
+        <v>457896</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3">
+        <v>2302</v>
+      </c>
+      <c r="K3" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3" t="s">
+        <v>29</v>
+      </c>
+      <c r="M3">
+        <v>4915110205551810</v>
+      </c>
+      <c r="N3" t="s">
+        <v>28</v>
+      </c>
+      <c r="O3">
+        <v>10016</v>
+      </c>
+      <c r="P3" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q3">
+        <v>3101234567</v>
+      </c>
+      <c r="R3">
+        <v>20000</v>
+      </c>
+      <c r="S3" t="s">
+        <v>31</v>
+      </c>
+      <c r="T3">
+        <v>1800</v>
+      </c>
+      <c r="U3" t="s">
+        <v>31</v>
+      </c>
+      <c r="V3" t="s">
+        <v>32</v>
+      </c>
+      <c r="W3">
+        <v>1245</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4">
+        <v>7946</v>
+      </c>
+      <c r="G4">
+        <v>6032</v>
+      </c>
+      <c r="H4">
+        <v>457896</v>
+      </c>
+      <c r="I4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4">
+        <v>2302</v>
+      </c>
+      <c r="K4" t="s">
+        <v>28</v>
+      </c>
+      <c r="L4" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4">
+        <v>4915110205551810</v>
+      </c>
+      <c r="N4" t="s">
+        <v>28</v>
+      </c>
+      <c r="O4">
+        <v>10016</v>
+      </c>
+      <c r="P4" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q4">
+        <v>3101234567</v>
+      </c>
+      <c r="R4">
+        <v>20000</v>
+      </c>
+      <c r="S4" t="s">
+        <v>31</v>
+      </c>
+      <c r="T4">
+        <v>1800</v>
+      </c>
+      <c r="U4" t="s">
+        <v>31</v>
+      </c>
+      <c r="V4" t="s">
+        <v>32</v>
+      </c>
+      <c r="W4">
+        <v>1245</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -926,7 +1075,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AC0694F-A5E4-46DE-ACB8-FCD5B5A7F1C2}">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
@@ -1089,6 +1238,74 @@
         <v>31</v>
       </c>
     </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3">
+        <v>7948</v>
+      </c>
+      <c r="G3">
+        <v>603237</v>
+      </c>
+      <c r="H3">
+        <v>184990</v>
+      </c>
+      <c r="I3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3">
+        <v>2302</v>
+      </c>
+      <c r="K3" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3">
+        <v>4473990520002990</v>
+      </c>
+      <c r="N3">
+        <v>15423459</v>
+      </c>
+      <c r="O3" t="s">
+        <v>28</v>
+      </c>
+      <c r="P3">
+        <v>10016</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>30</v>
+      </c>
+      <c r="R3">
+        <v>3118451263</v>
+      </c>
+      <c r="S3">
+        <v>20000</v>
+      </c>
+      <c r="T3" t="s">
+        <v>31</v>
+      </c>
+      <c r="U3">
+        <v>1800</v>
+      </c>
+      <c r="V3" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1096,353 +1313,802 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54C212FC-F1A9-4C3B-B367-0FC036FFD769}">
-  <dimension ref="A1:AV3"/>
+  <dimension ref="A1:AW5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="48.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="46.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="57.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="46.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="50.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="45.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="55.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="57.77734375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="53.77734375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="47.77734375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="71" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="51.77734375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="42.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="52.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="48.44140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="49.44140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="44.5546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="41.77734375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="52.88671875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="50.6640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="53.21875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="40.44140625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="45" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="38.5546875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="41.77734375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="41" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="51" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="53.44140625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="49.44140625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="66.6640625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="43.44140625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="38.21875" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="48.33203125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="39.109375" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="45.6640625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="50.109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="39.109375" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="45.6640625" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="50.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" customWidth="1"/>
+    <col min="3" max="3" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="53.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="52.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="48.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="46.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="57.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="46.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="50.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="45.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="48.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="55.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="57.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="53.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="47.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="71" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="51.77734375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="42.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="52.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="48.44140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="49.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="44.5546875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="41.77734375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="52.88671875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="50.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="53.21875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="40.44140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="45" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="38.5546875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="41.77734375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="41" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="51" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="53.44140625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="49.44140625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="66.6640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="43.44140625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="38.21875" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="48.33203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="39.109375" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="45.6640625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="50.109375" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="39.109375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="45.6640625" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="50.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:49" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:48" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
         <v>85</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>86</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2">
+        <v>7946</v>
+      </c>
+      <c r="F2">
+        <v>7946</v>
+      </c>
+      <c r="G2" t="s">
         <v>87</v>
       </c>
-      <c r="D2">
-        <v>7946</v>
-      </c>
-      <c r="E2">
-        <v>7946</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2">
+        <v>4594971</v>
+      </c>
+      <c r="J2">
+        <v>7946</v>
+      </c>
+      <c r="K2">
+        <v>123456789</v>
+      </c>
+      <c r="L2" t="s">
         <v>88</v>
       </c>
-      <c r="G2" t="s">
+      <c r="M2">
+        <v>12</v>
+      </c>
+      <c r="N2" t="s">
+        <v>89</v>
+      </c>
+      <c r="O2" t="s">
+        <v>90</v>
+      </c>
+      <c r="P2">
+        <v>1003214830</v>
+      </c>
+      <c r="Q2">
+        <v>7</v>
+      </c>
+      <c r="R2">
+        <v>10</v>
+      </c>
+      <c r="S2">
+        <v>1</v>
+      </c>
+      <c r="T2">
+        <v>11001</v>
+      </c>
+      <c r="U2" t="s">
+        <v>91</v>
+      </c>
+      <c r="V2" t="s">
+        <v>23</v>
+      </c>
+      <c r="W2" t="s">
+        <v>92</v>
+      </c>
+      <c r="X2">
+        <v>7946</v>
+      </c>
+      <c r="Y2">
+        <v>7946</v>
+      </c>
+      <c r="Z2">
+        <v>7946</v>
+      </c>
+      <c r="AA2" t="s">
         <v>25</v>
       </c>
-      <c r="H2">
+      <c r="AB2">
+        <v>4595976</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AE2">
+        <v>10000</v>
+      </c>
+      <c r="AF2">
+        <v>170</v>
+      </c>
+      <c r="AG2">
+        <v>12053337612</v>
+      </c>
+      <c r="AH2">
+        <v>7946</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>29</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AK2">
+        <v>821004207</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AM2">
+        <v>12053337612</v>
+      </c>
+      <c r="AN2">
+        <v>10</v>
+      </c>
+      <c r="AO2">
+        <v>7</v>
+      </c>
+      <c r="AP2">
+        <v>90025</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>95</v>
+      </c>
+      <c r="AS2">
+        <v>38020</v>
+      </c>
+      <c r="AT2">
+        <v>170</v>
+      </c>
+      <c r="AU2" t="s">
+        <v>96</v>
+      </c>
+      <c r="AV2">
+        <v>16520</v>
+      </c>
+      <c r="AW2">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:49" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3">
+        <v>7946</v>
+      </c>
+      <c r="F3">
+        <v>7946</v>
+      </c>
+      <c r="G3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3">
         <v>4594971</v>
       </c>
-      <c r="I2">
-        <v>7946</v>
-      </c>
-      <c r="J2">
+      <c r="J3">
+        <v>7946</v>
+      </c>
+      <c r="K3">
         <v>123456789</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L3" t="s">
+        <v>88</v>
+      </c>
+      <c r="M3">
+        <v>12</v>
+      </c>
+      <c r="N3" t="s">
         <v>89</v>
       </c>
-      <c r="L2">
+      <c r="O3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P3">
+        <v>1003214830</v>
+      </c>
+      <c r="Q3">
+        <v>7</v>
+      </c>
+      <c r="R3">
+        <v>10</v>
+      </c>
+      <c r="S3">
+        <v>1</v>
+      </c>
+      <c r="T3">
+        <v>11001</v>
+      </c>
+      <c r="U3" t="s">
+        <v>91</v>
+      </c>
+      <c r="V3" t="s">
+        <v>23</v>
+      </c>
+      <c r="W3" t="s">
+        <v>92</v>
+      </c>
+      <c r="X3">
+        <v>7946</v>
+      </c>
+      <c r="Y3">
+        <v>7946</v>
+      </c>
+      <c r="Z3">
+        <v>7946</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB3">
+        <v>4595976</v>
+      </c>
+      <c r="AC3" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>93</v>
+      </c>
+      <c r="AE3">
+        <v>10000</v>
+      </c>
+      <c r="AF3">
+        <v>170</v>
+      </c>
+      <c r="AG3">
+        <v>12053337612</v>
+      </c>
+      <c r="AH3">
+        <v>7946</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>94</v>
+      </c>
+      <c r="AK3">
+        <v>821004207</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>90</v>
+      </c>
+      <c r="AM3">
+        <v>12053337612</v>
+      </c>
+      <c r="AN3">
+        <v>10</v>
+      </c>
+      <c r="AO3">
+        <v>7</v>
+      </c>
+      <c r="AP3">
+        <v>90025</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>91</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>95</v>
+      </c>
+      <c r="AS3">
+        <v>38020</v>
+      </c>
+      <c r="AT3">
+        <v>170</v>
+      </c>
+      <c r="AU3" t="s">
+        <v>96</v>
+      </c>
+      <c r="AV3">
+        <v>16520</v>
+      </c>
+      <c r="AW3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:49" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4">
+        <v>7946</v>
+      </c>
+      <c r="F4">
+        <v>7946</v>
+      </c>
+      <c r="G4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4">
+        <v>4594971</v>
+      </c>
+      <c r="J4">
+        <v>7946</v>
+      </c>
+      <c r="K4">
+        <v>123456789</v>
+      </c>
+      <c r="L4" t="s">
+        <v>88</v>
+      </c>
+      <c r="M4">
         <v>12</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N4" t="s">
+        <v>89</v>
+      </c>
+      <c r="O4" t="s">
         <v>90</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P4">
+        <v>1003214830</v>
+      </c>
+      <c r="Q4">
+        <v>7</v>
+      </c>
+      <c r="R4">
+        <v>10</v>
+      </c>
+      <c r="S4">
+        <v>1</v>
+      </c>
+      <c r="T4">
+        <v>11001</v>
+      </c>
+      <c r="U4" t="s">
         <v>91</v>
       </c>
-      <c r="O2">
+      <c r="V4" t="s">
+        <v>23</v>
+      </c>
+      <c r="W4" t="s">
+        <v>92</v>
+      </c>
+      <c r="X4">
+        <v>7946</v>
+      </c>
+      <c r="Y4">
+        <v>7946</v>
+      </c>
+      <c r="Z4">
+        <v>7946</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB4">
+        <v>4595976</v>
+      </c>
+      <c r="AC4" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>93</v>
+      </c>
+      <c r="AE4">
+        <v>10000</v>
+      </c>
+      <c r="AF4">
+        <v>170</v>
+      </c>
+      <c r="AG4">
+        <v>12053337612</v>
+      </c>
+      <c r="AH4">
+        <v>7946</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>29</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>94</v>
+      </c>
+      <c r="AK4">
+        <v>821004207</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>90</v>
+      </c>
+      <c r="AM4">
+        <v>12053337612</v>
+      </c>
+      <c r="AN4">
+        <v>10</v>
+      </c>
+      <c r="AO4">
+        <v>7</v>
+      </c>
+      <c r="AP4">
+        <v>90025</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>91</v>
+      </c>
+      <c r="AR4" t="s">
+        <v>95</v>
+      </c>
+      <c r="AS4">
+        <v>38020</v>
+      </c>
+      <c r="AT4">
+        <v>170</v>
+      </c>
+      <c r="AU4" t="s">
+        <v>96</v>
+      </c>
+      <c r="AV4">
+        <v>16520</v>
+      </c>
+      <c r="AW4">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="5" spans="1:49" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5">
+        <v>7946</v>
+      </c>
+      <c r="F5">
+        <v>7946</v>
+      </c>
+      <c r="G5" t="s">
+        <v>87</v>
+      </c>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5">
+        <v>4594971</v>
+      </c>
+      <c r="J5">
+        <v>7946</v>
+      </c>
+      <c r="K5">
+        <v>123456789</v>
+      </c>
+      <c r="L5" t="s">
+        <v>88</v>
+      </c>
+      <c r="M5">
+        <v>12</v>
+      </c>
+      <c r="N5" t="s">
+        <v>89</v>
+      </c>
+      <c r="O5" t="s">
+        <v>90</v>
+      </c>
+      <c r="P5">
         <v>1003214830</v>
       </c>
-      <c r="P2">
+      <c r="Q5">
         <v>7</v>
       </c>
-      <c r="Q2">
+      <c r="R5">
         <v>10</v>
       </c>
-      <c r="R2">
+      <c r="S5">
         <v>1</v>
       </c>
-      <c r="S2">
+      <c r="T5">
         <v>11001</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U5" t="s">
+        <v>91</v>
+      </c>
+      <c r="V5" t="s">
+        <v>23</v>
+      </c>
+      <c r="W5" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="3" spans="1:48" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="X5">
+        <v>7946</v>
+      </c>
+      <c r="Y5">
+        <v>7946</v>
+      </c>
+      <c r="Z5">
+        <v>7946</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB5">
+        <v>4595976</v>
+      </c>
+      <c r="AC5" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="AD5" t="s">
         <v>93</v>
       </c>
-      <c r="U3" t="s">
-        <v>23</v>
-      </c>
-      <c r="V3" t="s">
+      <c r="AE5">
+        <v>10000</v>
+      </c>
+      <c r="AF5">
+        <v>170</v>
+      </c>
+      <c r="AG5">
+        <v>12053337612</v>
+      </c>
+      <c r="AH5">
+        <v>7946</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>29</v>
+      </c>
+      <c r="AJ5" t="s">
         <v>94</v>
       </c>
-      <c r="W3">
-        <v>7946</v>
-      </c>
-      <c r="X3">
-        <v>7946</v>
-      </c>
-      <c r="Y3">
-        <v>7946</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA3">
-        <v>4595976</v>
-      </c>
-      <c r="AB3">
-        <v>10002795130011</v>
-      </c>
-      <c r="AC3" t="s">
+      <c r="AK5">
+        <v>821004207</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>90</v>
+      </c>
+      <c r="AM5">
+        <v>12053337612</v>
+      </c>
+      <c r="AN5">
+        <v>10</v>
+      </c>
+      <c r="AO5">
+        <v>7</v>
+      </c>
+      <c r="AP5">
+        <v>90025</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>91</v>
+      </c>
+      <c r="AR5" t="s">
         <v>95</v>
       </c>
-      <c r="AD3">
-        <v>10000</v>
-      </c>
-      <c r="AE3">
+      <c r="AS5">
+        <v>38020</v>
+      </c>
+      <c r="AT5">
         <v>170</v>
       </c>
-      <c r="AF3">
-        <v>12053337612</v>
-      </c>
-      <c r="AG3">
-        <v>7946</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>29</v>
-      </c>
-      <c r="AI3" t="s">
+      <c r="AU5" t="s">
         <v>96</v>
       </c>
-      <c r="AJ3">
-        <v>821004207</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>91</v>
-      </c>
-      <c r="AL3">
-        <v>12053337612</v>
-      </c>
-      <c r="AM3">
-        <v>10</v>
-      </c>
-      <c r="AN3">
-        <v>7</v>
-      </c>
-      <c r="AO3">
-        <v>90025</v>
-      </c>
-      <c r="AP3" t="s">
-        <v>92</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>97</v>
-      </c>
-      <c r="AR3">
-        <v>38020</v>
-      </c>
-      <c r="AS3">
-        <v>170</v>
-      </c>
-      <c r="AT3" t="s">
-        <v>98</v>
-      </c>
-      <c r="AU3">
+      <c r="AV5">
         <v>16520</v>
       </c>
-      <c r="AV3">
+      <c r="AW5">
         <v>170</v>
       </c>
     </row>
@@ -1453,7 +2119,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1719BB12-E349-467A-982C-38FA62C753A4}">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
@@ -1505,31 +2171,31 @@
         <v>9</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -1537,7 +2203,7 @@
         <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C2" t="s">
         <v>25</v>
@@ -1579,12 +2245,68 @@
         <v>31</v>
       </c>
       <c r="P2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q2">
         <v>7946</v>
       </c>
       <c r="R2">
+        <v>4915110205551810</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3">
+        <v>7946</v>
+      </c>
+      <c r="G3">
+        <v>6032</v>
+      </c>
+      <c r="H3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3">
+        <v>2302</v>
+      </c>
+      <c r="J3" t="s">
+        <v>28</v>
+      </c>
+      <c r="K3" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3">
+        <v>2.0000010000089999E+23</v>
+      </c>
+      <c r="M3">
+        <v>10016</v>
+      </c>
+      <c r="N3">
+        <v>20000</v>
+      </c>
+      <c r="O3" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q3">
+        <v>7946</v>
+      </c>
+      <c r="R3">
         <v>4915110205551810</v>
       </c>
     </row>

</xml_diff>